<commit_message>
added functional groups to species list
</commit_message>
<xml_diff>
--- a/goa_efh_spp_lifestages.xlsx
+++ b/goa_efh_spp_lifestages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabellegalko/Documents/OSU/GOA CVA/Exposure/CVA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041E7FD7-7F6E-114F-AEC5-B39D98F38AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFFC223-B573-5F46-8585-3C73CE98F4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-13900" yWindow="-21680" windowWidth="21480" windowHeight="20340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="19000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="goa_efh_spp_lifestages" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="289">
   <si>
     <t>species</t>
   </si>
@@ -890,6 +890,21 @@
   </si>
   <si>
     <t xml:space="preserve">"Salmon_mature_Chum_efh_level1_distribution" </t>
+  </si>
+  <si>
+    <t>Flatfish</t>
+  </si>
+  <si>
+    <t>Elasmobranch</t>
+  </si>
+  <si>
+    <t>Rockfish</t>
+  </si>
+  <si>
+    <t>Groundfish</t>
+  </si>
+  <si>
+    <t>Mollusc</t>
   </si>
 </sst>
 </file>
@@ -3537,7 +3552,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <conditionalFormatting sqref="J3 D3:I8 D11:I14 D16:I16 D18:I18 D21:I21 D23:I23 D26:I26 D28:I30 D33:I33 D36:I38 D42:I48 D50:I52 D54:I54 D56:I1048576 J57 J38 J51 J11:J13">
+  <conditionalFormatting sqref="J3 D3:I8 J11:J13 D11:I14 D16:I16 D18:I18 D21:I21 D23:I23 D26:I26 D28:I30 D33:I33 D36:I38 J38 D42:I48 D50:I52 J51 D54:I54 D56:I1048576 J57">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="species">
       <formula>NOT(ISERROR(SEARCH("species",D3)))</formula>
     </cfRule>
@@ -3552,250 +3567,341 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D170607-8CD7-D247-BFB2-6FC2E88AB4B1}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="63.83203125" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="63.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" s="13" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C3" s="13" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C4" s="13" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>285</v>
+      </c>
+      <c r="B5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="C5" s="13" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>284</v>
+      </c>
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="C6" s="13" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>286</v>
+      </c>
+      <c r="B7" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="C7" s="13" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>284</v>
+      </c>
+      <c r="B8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="13" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>286</v>
+      </c>
+      <c r="B9" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="C9" s="13" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>285</v>
+      </c>
+      <c r="B10" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="13" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="C11" s="13" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>284</v>
+      </c>
+      <c r="B12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="C12" s="13" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>287</v>
+      </c>
+      <c r="B13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="C13" s="13" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>286</v>
+      </c>
+      <c r="B14" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="C14" s="13" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>284</v>
+      </c>
+      <c r="B15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="C15" s="13" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>286</v>
+      </c>
+      <c r="B16" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="C16" s="13" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>284</v>
+      </c>
+      <c r="B17" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="C17" s="13" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>286</v>
+      </c>
+      <c r="B18" t="s">
         <v>277</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="C18" s="13" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>287</v>
+      </c>
+      <c r="B19" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="C19" s="13" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>286</v>
+      </c>
+      <c r="B20" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="C20" s="13" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>286</v>
+      </c>
+      <c r="B21" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="C21" s="13" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>286</v>
+      </c>
+      <c r="B22" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="C22" s="13" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>286</v>
+      </c>
+      <c r="B23" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="C23" s="13" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>284</v>
+      </c>
+      <c r="B24" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="C24" s="13" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>285</v>
+      </c>
+      <c r="B25" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="C25" s="13" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>284</v>
+      </c>
+      <c r="B26" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="C26" s="13" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
+        <v>287</v>
+      </c>
+      <c r="B27" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="C27" s="13" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>286</v>
+      </c>
+      <c r="B28" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="C28" s="13" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>284</v>
+      </c>
+      <c r="B29" t="s">
         <v>18</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="C29" s="13" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>288</v>
+      </c>
+      <c r="B30" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="C30" s="13" t="s">
         <v>276</v>
       </c>
     </row>

</xml_diff>